<commit_message>
chore: update README metrics and density range to reflect additional dataset records
</commit_message>
<xml_diff>
--- a/Conversão da densidade observada para densidade a 20ºC/res-894-2022-01_pivot_format.xlsx
+++ b/Conversão da densidade observada para densidade a 20ºC/res-894-2022-01_pivot_format.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="840 a 849" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="850 a 859" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="860 a 869" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="870 a 879" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18575,4 +18576,3623 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K102"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Temp</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>0.870</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>0.871</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>0.872</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>0.873</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>0.874</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>0.875</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>0.876</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>0.877</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>0.878</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>0.879</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>0.8568</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>0.8578</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0.8589</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>0.8599</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>0.8609</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>0.8619</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>0.8629</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>0.8639</v>
+      </c>
+      <c r="J2" s="3" t="n">
+        <v>0.8649</v>
+      </c>
+      <c r="K2" s="3" t="n">
+        <v>0.8659</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>0.8572</v>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>0.8582</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>0.8592</v>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>0.8602</v>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>0.8612</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>0.8622</v>
+      </c>
+      <c r="H3" s="4" t="n">
+        <v>0.8632</v>
+      </c>
+      <c r="I3" s="4" t="n">
+        <v>0.8642</v>
+      </c>
+      <c r="J3" s="4" t="n">
+        <v>0.8653</v>
+      </c>
+      <c r="K3" s="4" t="n">
+        <v>0.8663</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0.8575</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>0.8585</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>0.8595</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>0.8605</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>0.8615</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>0.8626</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>0.8636</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>0.8646</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>0.8656</v>
+      </c>
+      <c r="K4" s="3" t="n">
+        <v>0.8666</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>0.8578</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>0.8588</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>0.8598</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>0.8609</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>0.8619</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>0.8629</v>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>0.8639</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>0.8649</v>
+      </c>
+      <c r="J5" s="4" t="n">
+        <v>0.8659</v>
+      </c>
+      <c r="K5" s="4" t="n">
+        <v>0.8669</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0.8582</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>0.8592</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>0.8602</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>0.8612</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>0.8622</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>0.8632</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>0.8642</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>0.8652</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>0.8662</v>
+      </c>
+      <c r="K6" s="3" t="n">
+        <v>0.8673</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>0.8585</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>0.8595</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>0.8605</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>0.8615</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>0.8625</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>0.8635</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>0.8646</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>0.8656</v>
+      </c>
+      <c r="J7" s="4" t="n">
+        <v>0.8666</v>
+      </c>
+      <c r="K7" s="4" t="n">
+        <v>0.8676</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>0.8588</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>0.8598</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>0.8609</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>0.8619</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>0.8629</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>0.8639</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>0.8649</v>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>0.8659</v>
+      </c>
+      <c r="J8" s="3" t="n">
+        <v>0.8669</v>
+      </c>
+      <c r="K8" s="3" t="n">
+        <v>0.8679</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>0.8592</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>0.8602</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>0.8612</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>0.8622</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>0.8632</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>0.8642</v>
+      </c>
+      <c r="H9" s="4" t="n">
+        <v>0.8652</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>0.8662</v>
+      </c>
+      <c r="J9" s="4" t="n">
+        <v>0.8672</v>
+      </c>
+      <c r="K9" s="4" t="n">
+        <v>0.8682</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0.8595</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>0.8605</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>0.8615</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>0.8625</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>0.8635</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>0.8645</v>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>0.8655</v>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>0.8666</v>
+      </c>
+      <c r="J10" s="3" t="n">
+        <v>0.8676</v>
+      </c>
+      <c r="K10" s="3" t="n">
+        <v>0.8686</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>0.8598</v>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>0.8608</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>0.8618</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>0.8629</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>0.8639</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>0.8649</v>
+      </c>
+      <c r="H11" s="4" t="n">
+        <v>0.8659</v>
+      </c>
+      <c r="I11" s="4" t="n">
+        <v>0.8669</v>
+      </c>
+      <c r="J11" s="4" t="n">
+        <v>0.8679</v>
+      </c>
+      <c r="K11" s="4" t="n">
+        <v>0.8689</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>0.8602</v>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>0.8612</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>0.8622</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>0.8632</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>0.8642</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>0.8652</v>
+      </c>
+      <c r="H12" s="3" t="n">
+        <v>0.8662</v>
+      </c>
+      <c r="I12" s="3" t="n">
+        <v>0.8672</v>
+      </c>
+      <c r="J12" s="3" t="n">
+        <v>0.8682</v>
+      </c>
+      <c r="K12" s="3" t="n">
+        <v>0.8692</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>0.8605</v>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>0.8615</v>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>0.8625</v>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>0.8635</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>0.8645</v>
+      </c>
+      <c r="G13" s="4" t="n">
+        <v>0.8655</v>
+      </c>
+      <c r="H13" s="4" t="n">
+        <v>0.8665</v>
+      </c>
+      <c r="I13" s="4" t="n">
+        <v>0.8675</v>
+      </c>
+      <c r="J13" s="4" t="n">
+        <v>0.8686</v>
+      </c>
+      <c r="K13" s="4" t="n">
+        <v>0.8696</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0.8608</v>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>0.8618</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>0.8628</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>0.8638</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>0.8649</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>0.8659</v>
+      </c>
+      <c r="H14" s="3" t="n">
+        <v>0.8669</v>
+      </c>
+      <c r="I14" s="3" t="n">
+        <v>0.8679</v>
+      </c>
+      <c r="J14" s="3" t="n">
+        <v>0.8689</v>
+      </c>
+      <c r="K14" s="3" t="n">
+        <v>0.8699</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="B15" s="4" t="n">
+        <v>0.8612</v>
+      </c>
+      <c r="C15" s="4" t="n">
+        <v>0.8622</v>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>0.8632</v>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>0.8642</v>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>0.8652</v>
+      </c>
+      <c r="G15" s="4" t="n">
+        <v>0.8662</v>
+      </c>
+      <c r="H15" s="4" t="n">
+        <v>0.8672</v>
+      </c>
+      <c r="I15" s="4" t="n">
+        <v>0.8682</v>
+      </c>
+      <c r="J15" s="4" t="n">
+        <v>0.8692</v>
+      </c>
+      <c r="K15" s="4" t="n">
+        <v>0.8702</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0.8615</v>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>0.8625</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>0.8635</v>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>0.8645</v>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>0.8655</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>0.8665</v>
+      </c>
+      <c r="H16" s="3" t="n">
+        <v>0.8675</v>
+      </c>
+      <c r="I16" s="3" t="n">
+        <v>0.8685</v>
+      </c>
+      <c r="J16" s="3" t="n">
+        <v>0.8695000000000001</v>
+      </c>
+      <c r="K16" s="3" t="n">
+        <v>0.8705000000000001</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="B17" s="4" t="n">
+        <v>0.8618</v>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>0.8628</v>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>0.8638</v>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>0.8648</v>
+      </c>
+      <c r="F17" s="4" t="n">
+        <v>0.8658</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>0.8668</v>
+      </c>
+      <c r="H17" s="4" t="n">
+        <v>0.8679</v>
+      </c>
+      <c r="I17" s="4" t="n">
+        <v>0.8689</v>
+      </c>
+      <c r="J17" s="4" t="n">
+        <v>0.8699</v>
+      </c>
+      <c r="K17" s="4" t="n">
+        <v>0.8709</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0.8621</v>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>0.8631</v>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>0.8642</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>0.8652</v>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>0.8662</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>0.8672</v>
+      </c>
+      <c r="H18" s="3" t="n">
+        <v>0.8682</v>
+      </c>
+      <c r="I18" s="3" t="n">
+        <v>0.8692</v>
+      </c>
+      <c r="J18" s="3" t="n">
+        <v>0.8702</v>
+      </c>
+      <c r="K18" s="3" t="n">
+        <v>0.8712</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>0.8625</v>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>0.8635</v>
+      </c>
+      <c r="D19" s="4" t="n">
+        <v>0.8645</v>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>0.8655</v>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>0.8665</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>0.8675</v>
+      </c>
+      <c r="H19" s="4" t="n">
+        <v>0.8685</v>
+      </c>
+      <c r="I19" s="4" t="n">
+        <v>0.8695000000000001</v>
+      </c>
+      <c r="J19" s="4" t="n">
+        <v>0.8705000000000001</v>
+      </c>
+      <c r="K19" s="4" t="n">
+        <v>0.8715000000000001</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0.8628</v>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>0.8638</v>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>0.8648</v>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>0.8658</v>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>0.8668</v>
+      </c>
+      <c r="G20" s="3" t="n">
+        <v>0.8678</v>
+      </c>
+      <c r="H20" s="3" t="n">
+        <v>0.8688</v>
+      </c>
+      <c r="I20" s="3" t="n">
+        <v>0.8698</v>
+      </c>
+      <c r="J20" s="3" t="n">
+        <v>0.8708</v>
+      </c>
+      <c r="K20" s="3" t="n">
+        <v>0.8719</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="B21" s="4" t="n">
+        <v>0.8631</v>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>0.8641</v>
+      </c>
+      <c r="D21" s="4" t="n">
+        <v>0.8651</v>
+      </c>
+      <c r="E21" s="4" t="n">
+        <v>0.8661</v>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>0.8672</v>
+      </c>
+      <c r="G21" s="4" t="n">
+        <v>0.8682</v>
+      </c>
+      <c r="H21" s="4" t="n">
+        <v>0.8692</v>
+      </c>
+      <c r="I21" s="4" t="n">
+        <v>0.8702</v>
+      </c>
+      <c r="J21" s="4" t="n">
+        <v>0.8712</v>
+      </c>
+      <c r="K21" s="4" t="n">
+        <v>0.8722</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0.8635</v>
+      </c>
+      <c r="C22" s="3" t="n">
+        <v>0.8645</v>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>0.8655</v>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>0.8665</v>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>0.8675</v>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>0.8685</v>
+      </c>
+      <c r="H22" s="3" t="n">
+        <v>0.8695000000000001</v>
+      </c>
+      <c r="I22" s="3" t="n">
+        <v>0.8705000000000001</v>
+      </c>
+      <c r="J22" s="3" t="n">
+        <v>0.8715000000000001</v>
+      </c>
+      <c r="K22" s="3" t="n">
+        <v>0.8725000000000001</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="B23" s="4" t="n">
+        <v>0.8638</v>
+      </c>
+      <c r="C23" s="4" t="n">
+        <v>0.8648</v>
+      </c>
+      <c r="D23" s="4" t="n">
+        <v>0.8658</v>
+      </c>
+      <c r="E23" s="4" t="n">
+        <v>0.8668</v>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>0.8678</v>
+      </c>
+      <c r="G23" s="4" t="n">
+        <v>0.8688</v>
+      </c>
+      <c r="H23" s="4" t="n">
+        <v>0.8698</v>
+      </c>
+      <c r="I23" s="4" t="n">
+        <v>0.8708</v>
+      </c>
+      <c r="J23" s="4" t="n">
+        <v>0.8718</v>
+      </c>
+      <c r="K23" s="4" t="n">
+        <v>0.8728</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0.8641</v>
+      </c>
+      <c r="C24" s="3" t="n">
+        <v>0.8651</v>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>0.8661</v>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>0.8671</v>
+      </c>
+      <c r="F24" s="3" t="n">
+        <v>0.8681</v>
+      </c>
+      <c r="G24" s="3" t="n">
+        <v>0.8691</v>
+      </c>
+      <c r="H24" s="3" t="n">
+        <v>0.8701</v>
+      </c>
+      <c r="I24" s="3" t="n">
+        <v>0.8711</v>
+      </c>
+      <c r="J24" s="3" t="n">
+        <v>0.8722</v>
+      </c>
+      <c r="K24" s="3" t="n">
+        <v>0.8732</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="B25" s="4" t="n">
+        <v>0.8643999999999999</v>
+      </c>
+      <c r="C25" s="4" t="n">
+        <v>0.8653999999999999</v>
+      </c>
+      <c r="D25" s="4" t="n">
+        <v>0.8665</v>
+      </c>
+      <c r="E25" s="4" t="n">
+        <v>0.8675</v>
+      </c>
+      <c r="F25" s="4" t="n">
+        <v>0.8685</v>
+      </c>
+      <c r="G25" s="4" t="n">
+        <v>0.8695000000000001</v>
+      </c>
+      <c r="H25" s="4" t="n">
+        <v>0.8705000000000001</v>
+      </c>
+      <c r="I25" s="4" t="n">
+        <v>0.8715000000000001</v>
+      </c>
+      <c r="J25" s="4" t="n">
+        <v>0.8725000000000001</v>
+      </c>
+      <c r="K25" s="4" t="n">
+        <v>0.8735000000000001</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0.8648</v>
+      </c>
+      <c r="C26" s="3" t="n">
+        <v>0.8658</v>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>0.8668</v>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>0.8678</v>
+      </c>
+      <c r="F26" s="3" t="n">
+        <v>0.8688</v>
+      </c>
+      <c r="G26" s="3" t="n">
+        <v>0.8698</v>
+      </c>
+      <c r="H26" s="3" t="n">
+        <v>0.8708</v>
+      </c>
+      <c r="I26" s="3" t="n">
+        <v>0.8718</v>
+      </c>
+      <c r="J26" s="3" t="n">
+        <v>0.8728</v>
+      </c>
+      <c r="K26" s="3" t="n">
+        <v>0.8738</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="B27" s="4" t="n">
+        <v>0.8651</v>
+      </c>
+      <c r="C27" s="4" t="n">
+        <v>0.8661</v>
+      </c>
+      <c r="D27" s="4" t="n">
+        <v>0.8671</v>
+      </c>
+      <c r="E27" s="4" t="n">
+        <v>0.8681</v>
+      </c>
+      <c r="F27" s="4" t="n">
+        <v>0.8691</v>
+      </c>
+      <c r="G27" s="4" t="n">
+        <v>0.8701</v>
+      </c>
+      <c r="H27" s="4" t="n">
+        <v>0.8711</v>
+      </c>
+      <c r="I27" s="4" t="n">
+        <v>0.8721</v>
+      </c>
+      <c r="J27" s="4" t="n">
+        <v>0.8731</v>
+      </c>
+      <c r="K27" s="4" t="n">
+        <v>0.8741</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>0.8653999999999999</v>
+      </c>
+      <c r="C28" s="3" t="n">
+        <v>0.8663999999999999</v>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>0.8673999999999999</v>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>0.8683999999999999</v>
+      </c>
+      <c r="F28" s="3" t="n">
+        <v>0.8694</v>
+      </c>
+      <c r="G28" s="3" t="n">
+        <v>0.8704</v>
+      </c>
+      <c r="H28" s="3" t="n">
+        <v>0.8714</v>
+      </c>
+      <c r="I28" s="3" t="n">
+        <v>0.8725000000000001</v>
+      </c>
+      <c r="J28" s="3" t="n">
+        <v>0.8735000000000001</v>
+      </c>
+      <c r="K28" s="3" t="n">
+        <v>0.8745000000000001</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="B29" s="4" t="n">
+        <v>0.8658</v>
+      </c>
+      <c r="C29" s="4" t="n">
+        <v>0.8668</v>
+      </c>
+      <c r="D29" s="4" t="n">
+        <v>0.8678</v>
+      </c>
+      <c r="E29" s="4" t="n">
+        <v>0.8688</v>
+      </c>
+      <c r="F29" s="4" t="n">
+        <v>0.8698</v>
+      </c>
+      <c r="G29" s="4" t="n">
+        <v>0.8708</v>
+      </c>
+      <c r="H29" s="4" t="n">
+        <v>0.8718</v>
+      </c>
+      <c r="I29" s="4" t="n">
+        <v>0.8728</v>
+      </c>
+      <c r="J29" s="4" t="n">
+        <v>0.8738</v>
+      </c>
+      <c r="K29" s="4" t="n">
+        <v>0.8748</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>0.8661</v>
+      </c>
+      <c r="C30" s="3" t="n">
+        <v>0.8671</v>
+      </c>
+      <c r="D30" s="3" t="n">
+        <v>0.8681</v>
+      </c>
+      <c r="E30" s="3" t="n">
+        <v>0.8691</v>
+      </c>
+      <c r="F30" s="3" t="n">
+        <v>0.8701</v>
+      </c>
+      <c r="G30" s="3" t="n">
+        <v>0.8711</v>
+      </c>
+      <c r="H30" s="3" t="n">
+        <v>0.8721</v>
+      </c>
+      <c r="I30" s="3" t="n">
+        <v>0.8731</v>
+      </c>
+      <c r="J30" s="3" t="n">
+        <v>0.8741</v>
+      </c>
+      <c r="K30" s="3" t="n">
+        <v>0.8751</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="B31" s="4" t="n">
+        <v>0.8663999999999999</v>
+      </c>
+      <c r="C31" s="4" t="n">
+        <v>0.8673999999999999</v>
+      </c>
+      <c r="D31" s="4" t="n">
+        <v>0.8683999999999999</v>
+      </c>
+      <c r="E31" s="4" t="n">
+        <v>0.8694</v>
+      </c>
+      <c r="F31" s="4" t="n">
+        <v>0.8704</v>
+      </c>
+      <c r="G31" s="4" t="n">
+        <v>0.8714</v>
+      </c>
+      <c r="H31" s="4" t="n">
+        <v>0.8724</v>
+      </c>
+      <c r="I31" s="4" t="n">
+        <v>0.8734</v>
+      </c>
+      <c r="J31" s="4" t="n">
+        <v>0.8744</v>
+      </c>
+      <c r="K31" s="4" t="n">
+        <v>0.8754</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0.8667</v>
+      </c>
+      <c r="C32" s="3" t="n">
+        <v>0.8677</v>
+      </c>
+      <c r="D32" s="3" t="n">
+        <v>0.8687</v>
+      </c>
+      <c r="E32" s="3" t="n">
+        <v>0.8697</v>
+      </c>
+      <c r="F32" s="3" t="n">
+        <v>0.8707</v>
+      </c>
+      <c r="G32" s="3" t="n">
+        <v>0.8717</v>
+      </c>
+      <c r="H32" s="3" t="n">
+        <v>0.8727</v>
+      </c>
+      <c r="I32" s="3" t="n">
+        <v>0.8738</v>
+      </c>
+      <c r="J32" s="3" t="n">
+        <v>0.8748</v>
+      </c>
+      <c r="K32" s="3" t="n">
+        <v>0.8758</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="B33" s="4" t="n">
+        <v>0.8671</v>
+      </c>
+      <c r="C33" s="4" t="n">
+        <v>0.8681</v>
+      </c>
+      <c r="D33" s="4" t="n">
+        <v>0.8691</v>
+      </c>
+      <c r="E33" s="4" t="n">
+        <v>0.8701</v>
+      </c>
+      <c r="F33" s="4" t="n">
+        <v>0.8711</v>
+      </c>
+      <c r="G33" s="4" t="n">
+        <v>0.8721</v>
+      </c>
+      <c r="H33" s="4" t="n">
+        <v>0.8731</v>
+      </c>
+      <c r="I33" s="4" t="n">
+        <v>0.8741</v>
+      </c>
+      <c r="J33" s="4" t="n">
+        <v>0.8751</v>
+      </c>
+      <c r="K33" s="4" t="n">
+        <v>0.8761</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>0.8673999999999999</v>
+      </c>
+      <c r="C34" s="3" t="n">
+        <v>0.8683999999999999</v>
+      </c>
+      <c r="D34" s="3" t="n">
+        <v>0.8694</v>
+      </c>
+      <c r="E34" s="3" t="n">
+        <v>0.8704</v>
+      </c>
+      <c r="F34" s="3" t="n">
+        <v>0.8714</v>
+      </c>
+      <c r="G34" s="3" t="n">
+        <v>0.8724</v>
+      </c>
+      <c r="H34" s="3" t="n">
+        <v>0.8734</v>
+      </c>
+      <c r="I34" s="3" t="n">
+        <v>0.8744</v>
+      </c>
+      <c r="J34" s="3" t="n">
+        <v>0.8754</v>
+      </c>
+      <c r="K34" s="3" t="n">
+        <v>0.8764</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="B35" s="4" t="n">
+        <v>0.8677</v>
+      </c>
+      <c r="C35" s="4" t="n">
+        <v>0.8687</v>
+      </c>
+      <c r="D35" s="4" t="n">
+        <v>0.8697</v>
+      </c>
+      <c r="E35" s="4" t="n">
+        <v>0.8707</v>
+      </c>
+      <c r="F35" s="4" t="n">
+        <v>0.8717</v>
+      </c>
+      <c r="G35" s="4" t="n">
+        <v>0.8727</v>
+      </c>
+      <c r="H35" s="4" t="n">
+        <v>0.8737</v>
+      </c>
+      <c r="I35" s="4" t="n">
+        <v>0.8747</v>
+      </c>
+      <c r="J35" s="4" t="n">
+        <v>0.8757</v>
+      </c>
+      <c r="K35" s="4" t="n">
+        <v>0.8767</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0.868</v>
+      </c>
+      <c r="C36" s="3" t="n">
+        <v>0.869</v>
+      </c>
+      <c r="D36" s="3" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="E36" s="3" t="n">
+        <v>0.871</v>
+      </c>
+      <c r="F36" s="3" t="n">
+        <v>0.8721</v>
+      </c>
+      <c r="G36" s="3" t="n">
+        <v>0.8731</v>
+      </c>
+      <c r="H36" s="3" t="n">
+        <v>0.8741</v>
+      </c>
+      <c r="I36" s="3" t="n">
+        <v>0.8751</v>
+      </c>
+      <c r="J36" s="3" t="n">
+        <v>0.8761</v>
+      </c>
+      <c r="K36" s="3" t="n">
+        <v>0.8771</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="B37" s="4" t="n">
+        <v>0.8683999999999999</v>
+      </c>
+      <c r="C37" s="4" t="n">
+        <v>0.8694</v>
+      </c>
+      <c r="D37" s="4" t="n">
+        <v>0.8704</v>
+      </c>
+      <c r="E37" s="4" t="n">
+        <v>0.8714</v>
+      </c>
+      <c r="F37" s="4" t="n">
+        <v>0.8724</v>
+      </c>
+      <c r="G37" s="4" t="n">
+        <v>0.8734</v>
+      </c>
+      <c r="H37" s="4" t="n">
+        <v>0.8744</v>
+      </c>
+      <c r="I37" s="4" t="n">
+        <v>0.8754</v>
+      </c>
+      <c r="J37" s="4" t="n">
+        <v>0.8764</v>
+      </c>
+      <c r="K37" s="4" t="n">
+        <v>0.8774</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>0.8687</v>
+      </c>
+      <c r="C38" s="3" t="n">
+        <v>0.8697</v>
+      </c>
+      <c r="D38" s="3" t="n">
+        <v>0.8707</v>
+      </c>
+      <c r="E38" s="3" t="n">
+        <v>0.8717</v>
+      </c>
+      <c r="F38" s="3" t="n">
+        <v>0.8727</v>
+      </c>
+      <c r="G38" s="3" t="n">
+        <v>0.8737</v>
+      </c>
+      <c r="H38" s="3" t="n">
+        <v>0.8747</v>
+      </c>
+      <c r="I38" s="3" t="n">
+        <v>0.8757</v>
+      </c>
+      <c r="J38" s="3" t="n">
+        <v>0.8767</v>
+      </c>
+      <c r="K38" s="3" t="n">
+        <v>0.8777</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="B39" s="4" t="n">
+        <v>0.869</v>
+      </c>
+      <c r="C39" s="4" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="D39" s="4" t="n">
+        <v>0.871</v>
+      </c>
+      <c r="E39" s="4" t="n">
+        <v>0.872</v>
+      </c>
+      <c r="F39" s="4" t="n">
+        <v>0.873</v>
+      </c>
+      <c r="G39" s="4" t="n">
+        <v>0.874</v>
+      </c>
+      <c r="H39" s="4" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="I39" s="4" t="n">
+        <v>0.876</v>
+      </c>
+      <c r="J39" s="4" t="n">
+        <v>0.877</v>
+      </c>
+      <c r="K39" s="4" t="n">
+        <v>0.878</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>0.8693</v>
+      </c>
+      <c r="C40" s="3" t="n">
+        <v>0.8704</v>
+      </c>
+      <c r="D40" s="3" t="n">
+        <v>0.8714</v>
+      </c>
+      <c r="E40" s="3" t="n">
+        <v>0.8724</v>
+      </c>
+      <c r="F40" s="3" t="n">
+        <v>0.8734</v>
+      </c>
+      <c r="G40" s="3" t="n">
+        <v>0.8744</v>
+      </c>
+      <c r="H40" s="3" t="n">
+        <v>0.8754</v>
+      </c>
+      <c r="I40" s="3" t="n">
+        <v>0.8764</v>
+      </c>
+      <c r="J40" s="3" t="n">
+        <v>0.8774</v>
+      </c>
+      <c r="K40" s="3" t="n">
+        <v>0.8784</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="B41" s="4" t="n">
+        <v>0.8697</v>
+      </c>
+      <c r="C41" s="4" t="n">
+        <v>0.8707</v>
+      </c>
+      <c r="D41" s="4" t="n">
+        <v>0.8717</v>
+      </c>
+      <c r="E41" s="4" t="n">
+        <v>0.8727</v>
+      </c>
+      <c r="F41" s="4" t="n">
+        <v>0.8737</v>
+      </c>
+      <c r="G41" s="4" t="n">
+        <v>0.8747</v>
+      </c>
+      <c r="H41" s="4" t="n">
+        <v>0.8757</v>
+      </c>
+      <c r="I41" s="4" t="n">
+        <v>0.8767</v>
+      </c>
+      <c r="J41" s="4" t="n">
+        <v>0.8777</v>
+      </c>
+      <c r="K41" s="4" t="n">
+        <v>0.8787</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="C42" s="3" t="n">
+        <v>0.871</v>
+      </c>
+      <c r="D42" s="3" t="n">
+        <v>0.872</v>
+      </c>
+      <c r="E42" s="3" t="n">
+        <v>0.873</v>
+      </c>
+      <c r="F42" s="3" t="n">
+        <v>0.874</v>
+      </c>
+      <c r="G42" s="3" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="H42" s="3" t="n">
+        <v>0.876</v>
+      </c>
+      <c r="I42" s="3" t="n">
+        <v>0.877</v>
+      </c>
+      <c r="J42" s="3" t="n">
+        <v>0.878</v>
+      </c>
+      <c r="K42" s="3" t="n">
+        <v>0.879</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="B43" s="4" t="n">
+        <v>0.8703</v>
+      </c>
+      <c r="C43" s="4" t="n">
+        <v>0.8713</v>
+      </c>
+      <c r="D43" s="4" t="n">
+        <v>0.8723</v>
+      </c>
+      <c r="E43" s="4" t="n">
+        <v>0.8733</v>
+      </c>
+      <c r="F43" s="4" t="n">
+        <v>0.8743</v>
+      </c>
+      <c r="G43" s="4" t="n">
+        <v>0.8753</v>
+      </c>
+      <c r="H43" s="4" t="n">
+        <v>0.8763</v>
+      </c>
+      <c r="I43" s="4" t="n">
+        <v>0.8773</v>
+      </c>
+      <c r="J43" s="4" t="n">
+        <v>0.8783</v>
+      </c>
+      <c r="K43" s="4" t="n">
+        <v>0.8793</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0.8706</v>
+      </c>
+      <c r="C44" s="3" t="n">
+        <v>0.8716</v>
+      </c>
+      <c r="D44" s="3" t="n">
+        <v>0.8726</v>
+      </c>
+      <c r="E44" s="3" t="n">
+        <v>0.8736</v>
+      </c>
+      <c r="F44" s="3" t="n">
+        <v>0.8746</v>
+      </c>
+      <c r="G44" s="3" t="n">
+        <v>0.8756</v>
+      </c>
+      <c r="H44" s="3" t="n">
+        <v>0.8766</v>
+      </c>
+      <c r="I44" s="3" t="n">
+        <v>0.8776</v>
+      </c>
+      <c r="J44" s="3" t="n">
+        <v>0.8786</v>
+      </c>
+      <c r="K44" s="3" t="n">
+        <v>0.8796</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="B45" s="4" t="n">
+        <v>0.871</v>
+      </c>
+      <c r="C45" s="4" t="n">
+        <v>0.872</v>
+      </c>
+      <c r="D45" s="4" t="n">
+        <v>0.873</v>
+      </c>
+      <c r="E45" s="4" t="n">
+        <v>0.874</v>
+      </c>
+      <c r="F45" s="4" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G45" s="4" t="n">
+        <v>0.876</v>
+      </c>
+      <c r="H45" s="4" t="n">
+        <v>0.877</v>
+      </c>
+      <c r="I45" s="4" t="n">
+        <v>0.878</v>
+      </c>
+      <c r="J45" s="4" t="n">
+        <v>0.879</v>
+      </c>
+      <c r="K45" s="4" t="n">
+        <v>0.88</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0.8713</v>
+      </c>
+      <c r="C46" s="3" t="n">
+        <v>0.8723</v>
+      </c>
+      <c r="D46" s="3" t="n">
+        <v>0.8733</v>
+      </c>
+      <c r="E46" s="3" t="n">
+        <v>0.8743</v>
+      </c>
+      <c r="F46" s="3" t="n">
+        <v>0.8753</v>
+      </c>
+      <c r="G46" s="3" t="n">
+        <v>0.8763</v>
+      </c>
+      <c r="H46" s="3" t="n">
+        <v>0.8773</v>
+      </c>
+      <c r="I46" s="3" t="n">
+        <v>0.8783</v>
+      </c>
+      <c r="J46" s="3" t="n">
+        <v>0.8793</v>
+      </c>
+      <c r="K46" s="3" t="n">
+        <v>0.8803</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="B47" s="4" t="n">
+        <v>0.8716</v>
+      </c>
+      <c r="C47" s="4" t="n">
+        <v>0.8726</v>
+      </c>
+      <c r="D47" s="4" t="n">
+        <v>0.8736</v>
+      </c>
+      <c r="E47" s="4" t="n">
+        <v>0.8746</v>
+      </c>
+      <c r="F47" s="4" t="n">
+        <v>0.8756</v>
+      </c>
+      <c r="G47" s="4" t="n">
+        <v>0.8766</v>
+      </c>
+      <c r="H47" s="4" t="n">
+        <v>0.8776</v>
+      </c>
+      <c r="I47" s="4" t="n">
+        <v>0.8786</v>
+      </c>
+      <c r="J47" s="4" t="n">
+        <v>0.8796</v>
+      </c>
+      <c r="K47" s="4" t="n">
+        <v>0.8806</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>0.8719</v>
+      </c>
+      <c r="C48" s="3" t="n">
+        <v>0.8729</v>
+      </c>
+      <c r="D48" s="3" t="n">
+        <v>0.8739</v>
+      </c>
+      <c r="E48" s="3" t="n">
+        <v>0.8749</v>
+      </c>
+      <c r="F48" s="3" t="n">
+        <v>0.8759</v>
+      </c>
+      <c r="G48" s="3" t="n">
+        <v>0.8769</v>
+      </c>
+      <c r="H48" s="3" t="n">
+        <v>0.8779</v>
+      </c>
+      <c r="I48" s="3" t="n">
+        <v>0.8789</v>
+      </c>
+      <c r="J48" s="3" t="n">
+        <v>0.8799</v>
+      </c>
+      <c r="K48" s="3" t="n">
+        <v>0.8809</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="B49" s="4" t="n">
+        <v>0.8723</v>
+      </c>
+      <c r="C49" s="4" t="n">
+        <v>0.8733</v>
+      </c>
+      <c r="D49" s="4" t="n">
+        <v>0.8743</v>
+      </c>
+      <c r="E49" s="4" t="n">
+        <v>0.8753</v>
+      </c>
+      <c r="F49" s="4" t="n">
+        <v>0.8763</v>
+      </c>
+      <c r="G49" s="4" t="n">
+        <v>0.8772</v>
+      </c>
+      <c r="H49" s="4" t="n">
+        <v>0.8782</v>
+      </c>
+      <c r="I49" s="4" t="n">
+        <v>0.8792</v>
+      </c>
+      <c r="J49" s="4" t="n">
+        <v>0.8802</v>
+      </c>
+      <c r="K49" s="4" t="n">
+        <v>0.8812</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>0.8726</v>
+      </c>
+      <c r="C50" s="3" t="n">
+        <v>0.8736</v>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>0.8746</v>
+      </c>
+      <c r="E50" s="3" t="n">
+        <v>0.8756</v>
+      </c>
+      <c r="F50" s="3" t="n">
+        <v>0.8766</v>
+      </c>
+      <c r="G50" s="3" t="n">
+        <v>0.8776</v>
+      </c>
+      <c r="H50" s="3" t="n">
+        <v>0.8786</v>
+      </c>
+      <c r="I50" s="3" t="n">
+        <v>0.8796</v>
+      </c>
+      <c r="J50" s="3" t="n">
+        <v>0.8806</v>
+      </c>
+      <c r="K50" s="3" t="n">
+        <v>0.8816000000000001</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="B51" s="4" t="n">
+        <v>0.8729</v>
+      </c>
+      <c r="C51" s="4" t="n">
+        <v>0.8739</v>
+      </c>
+      <c r="D51" s="4" t="n">
+        <v>0.8749</v>
+      </c>
+      <c r="E51" s="4" t="n">
+        <v>0.8759</v>
+      </c>
+      <c r="F51" s="4" t="n">
+        <v>0.8769</v>
+      </c>
+      <c r="G51" s="4" t="n">
+        <v>0.8779</v>
+      </c>
+      <c r="H51" s="4" t="n">
+        <v>0.8789</v>
+      </c>
+      <c r="I51" s="4" t="n">
+        <v>0.8799</v>
+      </c>
+      <c r="J51" s="4" t="n">
+        <v>0.8809</v>
+      </c>
+      <c r="K51" s="4" t="n">
+        <v>0.8819</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>0.8732</v>
+      </c>
+      <c r="C52" s="3" t="n">
+        <v>0.8742</v>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>0.8752</v>
+      </c>
+      <c r="E52" s="3" t="n">
+        <v>0.8762</v>
+      </c>
+      <c r="F52" s="3" t="n">
+        <v>0.8772</v>
+      </c>
+      <c r="G52" s="3" t="n">
+        <v>0.8782</v>
+      </c>
+      <c r="H52" s="3" t="n">
+        <v>0.8792</v>
+      </c>
+      <c r="I52" s="3" t="n">
+        <v>0.8802</v>
+      </c>
+      <c r="J52" s="3" t="n">
+        <v>0.8812</v>
+      </c>
+      <c r="K52" s="3" t="n">
+        <v>0.8822</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="B53" s="4" t="n">
+        <v>0.8735000000000001</v>
+      </c>
+      <c r="C53" s="4" t="n">
+        <v>0.8745000000000001</v>
+      </c>
+      <c r="D53" s="4" t="n">
+        <v>0.8754999999999999</v>
+      </c>
+      <c r="E53" s="4" t="n">
+        <v>0.8764999999999999</v>
+      </c>
+      <c r="F53" s="4" t="n">
+        <v>0.8774999999999999</v>
+      </c>
+      <c r="G53" s="4" t="n">
+        <v>0.8784999999999999</v>
+      </c>
+      <c r="H53" s="4" t="n">
+        <v>0.8794999999999999</v>
+      </c>
+      <c r="I53" s="4" t="n">
+        <v>0.8804999999999999</v>
+      </c>
+      <c r="J53" s="4" t="n">
+        <v>0.8815</v>
+      </c>
+      <c r="K53" s="4" t="n">
+        <v>0.8825</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>0.8739</v>
+      </c>
+      <c r="C54" s="3" t="n">
+        <v>0.8749</v>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>0.8759</v>
+      </c>
+      <c r="E54" s="3" t="n">
+        <v>0.8769</v>
+      </c>
+      <c r="F54" s="3" t="n">
+        <v>0.8779</v>
+      </c>
+      <c r="G54" s="3" t="n">
+        <v>0.8789</v>
+      </c>
+      <c r="H54" s="3" t="n">
+        <v>0.8799</v>
+      </c>
+      <c r="I54" s="3" t="n">
+        <v>0.8809</v>
+      </c>
+      <c r="J54" s="3" t="n">
+        <v>0.8819</v>
+      </c>
+      <c r="K54" s="3" t="n">
+        <v>0.8829</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="B55" s="4" t="n">
+        <v>0.8742</v>
+      </c>
+      <c r="C55" s="4" t="n">
+        <v>0.8752</v>
+      </c>
+      <c r="D55" s="4" t="n">
+        <v>0.8762</v>
+      </c>
+      <c r="E55" s="4" t="n">
+        <v>0.8772</v>
+      </c>
+      <c r="F55" s="4" t="n">
+        <v>0.8782</v>
+      </c>
+      <c r="G55" s="4" t="n">
+        <v>0.8792</v>
+      </c>
+      <c r="H55" s="4" t="n">
+        <v>0.8802</v>
+      </c>
+      <c r="I55" s="4" t="n">
+        <v>0.8812</v>
+      </c>
+      <c r="J55" s="4" t="n">
+        <v>0.8822</v>
+      </c>
+      <c r="K55" s="4" t="n">
+        <v>0.8832</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0.8745000000000001</v>
+      </c>
+      <c r="C56" s="3" t="n">
+        <v>0.8754999999999999</v>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>0.8764999999999999</v>
+      </c>
+      <c r="E56" s="3" t="n">
+        <v>0.8774999999999999</v>
+      </c>
+      <c r="F56" s="3" t="n">
+        <v>0.8784999999999999</v>
+      </c>
+      <c r="G56" s="3" t="n">
+        <v>0.8794999999999999</v>
+      </c>
+      <c r="H56" s="3" t="n">
+        <v>0.8804999999999999</v>
+      </c>
+      <c r="I56" s="3" t="n">
+        <v>0.8815</v>
+      </c>
+      <c r="J56" s="3" t="n">
+        <v>0.8825</v>
+      </c>
+      <c r="K56" s="3" t="n">
+        <v>0.8835</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="B57" s="4" t="n">
+        <v>0.8748</v>
+      </c>
+      <c r="C57" s="4" t="n">
+        <v>0.8758</v>
+      </c>
+      <c r="D57" s="4" t="n">
+        <v>0.8768</v>
+      </c>
+      <c r="E57" s="4" t="n">
+        <v>0.8778</v>
+      </c>
+      <c r="F57" s="4" t="n">
+        <v>0.8788</v>
+      </c>
+      <c r="G57" s="4" t="n">
+        <v>0.8798</v>
+      </c>
+      <c r="H57" s="4" t="n">
+        <v>0.8808</v>
+      </c>
+      <c r="I57" s="4" t="n">
+        <v>0.8818</v>
+      </c>
+      <c r="J57" s="4" t="n">
+        <v>0.8828</v>
+      </c>
+      <c r="K57" s="4" t="n">
+        <v>0.8838</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>0.8752</v>
+      </c>
+      <c r="C58" s="3" t="n">
+        <v>0.8762</v>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>0.8772</v>
+      </c>
+      <c r="E58" s="3" t="n">
+        <v>0.8781</v>
+      </c>
+      <c r="F58" s="3" t="n">
+        <v>0.8791</v>
+      </c>
+      <c r="G58" s="3" t="n">
+        <v>0.8801</v>
+      </c>
+      <c r="H58" s="3" t="n">
+        <v>0.8811</v>
+      </c>
+      <c r="I58" s="3" t="n">
+        <v>0.8821</v>
+      </c>
+      <c r="J58" s="3" t="n">
+        <v>0.8831</v>
+      </c>
+      <c r="K58" s="3" t="n">
+        <v>0.8841</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="B59" s="4" t="n">
+        <v>0.8754999999999999</v>
+      </c>
+      <c r="C59" s="4" t="n">
+        <v>0.8764999999999999</v>
+      </c>
+      <c r="D59" s="4" t="n">
+        <v>0.8774999999999999</v>
+      </c>
+      <c r="E59" s="4" t="n">
+        <v>0.8784999999999999</v>
+      </c>
+      <c r="F59" s="4" t="n">
+        <v>0.8794999999999999</v>
+      </c>
+      <c r="G59" s="4" t="n">
+        <v>0.8804999999999999</v>
+      </c>
+      <c r="H59" s="4" t="n">
+        <v>0.8815</v>
+      </c>
+      <c r="I59" s="4" t="n">
+        <v>0.8825</v>
+      </c>
+      <c r="J59" s="4" t="n">
+        <v>0.8835</v>
+      </c>
+      <c r="K59" s="4" t="n">
+        <v>0.8845</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B60" s="3" t="n">
+        <v>0.8758</v>
+      </c>
+      <c r="C60" s="3" t="n">
+        <v>0.8768</v>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>0.8778</v>
+      </c>
+      <c r="E60" s="3" t="n">
+        <v>0.8788</v>
+      </c>
+      <c r="F60" s="3" t="n">
+        <v>0.8798</v>
+      </c>
+      <c r="G60" s="3" t="n">
+        <v>0.8808</v>
+      </c>
+      <c r="H60" s="3" t="n">
+        <v>0.8818</v>
+      </c>
+      <c r="I60" s="3" t="n">
+        <v>0.8828</v>
+      </c>
+      <c r="J60" s="3" t="n">
+        <v>0.8838</v>
+      </c>
+      <c r="K60" s="3" t="n">
+        <v>0.8848</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="B61" s="4" t="n">
+        <v>0.8761</v>
+      </c>
+      <c r="C61" s="4" t="n">
+        <v>0.8771</v>
+      </c>
+      <c r="D61" s="4" t="n">
+        <v>0.8781</v>
+      </c>
+      <c r="E61" s="4" t="n">
+        <v>0.8791</v>
+      </c>
+      <c r="F61" s="4" t="n">
+        <v>0.8801</v>
+      </c>
+      <c r="G61" s="4" t="n">
+        <v>0.8811</v>
+      </c>
+      <c r="H61" s="4" t="n">
+        <v>0.8821</v>
+      </c>
+      <c r="I61" s="4" t="n">
+        <v>0.8831</v>
+      </c>
+      <c r="J61" s="4" t="n">
+        <v>0.8841</v>
+      </c>
+      <c r="K61" s="4" t="n">
+        <v>0.8851</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B62" s="3" t="n">
+        <v>0.8764</v>
+      </c>
+      <c r="C62" s="3" t="n">
+        <v>0.8774</v>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>0.8784</v>
+      </c>
+      <c r="E62" s="3" t="n">
+        <v>0.8794</v>
+      </c>
+      <c r="F62" s="3" t="n">
+        <v>0.8804</v>
+      </c>
+      <c r="G62" s="3" t="n">
+        <v>0.8814</v>
+      </c>
+      <c r="H62" s="3" t="n">
+        <v>0.8824</v>
+      </c>
+      <c r="I62" s="3" t="n">
+        <v>0.8834</v>
+      </c>
+      <c r="J62" s="3" t="n">
+        <v>0.8844</v>
+      </c>
+      <c r="K62" s="3" t="n">
+        <v>0.8854</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="B63" s="4" t="n">
+        <v>0.8768</v>
+      </c>
+      <c r="C63" s="4" t="n">
+        <v>0.8778</v>
+      </c>
+      <c r="D63" s="4" t="n">
+        <v>0.8788</v>
+      </c>
+      <c r="E63" s="4" t="n">
+        <v>0.8798</v>
+      </c>
+      <c r="F63" s="4" t="n">
+        <v>0.8807</v>
+      </c>
+      <c r="G63" s="4" t="n">
+        <v>0.8817</v>
+      </c>
+      <c r="H63" s="4" t="n">
+        <v>0.8827</v>
+      </c>
+      <c r="I63" s="4" t="n">
+        <v>0.8837</v>
+      </c>
+      <c r="J63" s="4" t="n">
+        <v>0.8847</v>
+      </c>
+      <c r="K63" s="4" t="n">
+        <v>0.8857</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B64" s="3" t="n">
+        <v>0.8771</v>
+      </c>
+      <c r="C64" s="3" t="n">
+        <v>0.8781</v>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>0.8791</v>
+      </c>
+      <c r="E64" s="3" t="n">
+        <v>0.8801</v>
+      </c>
+      <c r="F64" s="3" t="n">
+        <v>0.8811</v>
+      </c>
+      <c r="G64" s="3" t="n">
+        <v>0.8821</v>
+      </c>
+      <c r="H64" s="3" t="n">
+        <v>0.8831</v>
+      </c>
+      <c r="I64" s="3" t="n">
+        <v>0.8841</v>
+      </c>
+      <c r="J64" s="3" t="n">
+        <v>0.8851</v>
+      </c>
+      <c r="K64" s="3" t="n">
+        <v>0.886</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="B65" s="4" t="n">
+        <v>0.8774</v>
+      </c>
+      <c r="C65" s="4" t="n">
+        <v>0.8784</v>
+      </c>
+      <c r="D65" s="4" t="n">
+        <v>0.8794</v>
+      </c>
+      <c r="E65" s="4" t="n">
+        <v>0.8804</v>
+      </c>
+      <c r="F65" s="4" t="n">
+        <v>0.8814</v>
+      </c>
+      <c r="G65" s="4" t="n">
+        <v>0.8824</v>
+      </c>
+      <c r="H65" s="4" t="n">
+        <v>0.8834</v>
+      </c>
+      <c r="I65" s="4" t="n">
+        <v>0.8844</v>
+      </c>
+      <c r="J65" s="4" t="n">
+        <v>0.8854</v>
+      </c>
+      <c r="K65" s="4" t="n">
+        <v>0.8864</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="B66" s="3" t="n">
+        <v>0.8777</v>
+      </c>
+      <c r="C66" s="3" t="n">
+        <v>0.8787</v>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>0.8797</v>
+      </c>
+      <c r="E66" s="3" t="n">
+        <v>0.8807</v>
+      </c>
+      <c r="F66" s="3" t="n">
+        <v>0.8817</v>
+      </c>
+      <c r="G66" s="3" t="n">
+        <v>0.8827</v>
+      </c>
+      <c r="H66" s="3" t="n">
+        <v>0.8837</v>
+      </c>
+      <c r="I66" s="3" t="n">
+        <v>0.8847</v>
+      </c>
+      <c r="J66" s="3" t="n">
+        <v>0.8857</v>
+      </c>
+      <c r="K66" s="3" t="n">
+        <v>0.8867</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="B67" s="4" t="n">
+        <v>0.878</v>
+      </c>
+      <c r="C67" s="4" t="n">
+        <v>0.879</v>
+      </c>
+      <c r="D67" s="4" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="E67" s="4" t="n">
+        <v>0.881</v>
+      </c>
+      <c r="F67" s="4" t="n">
+        <v>0.882</v>
+      </c>
+      <c r="G67" s="4" t="n">
+        <v>0.883</v>
+      </c>
+      <c r="H67" s="4" t="n">
+        <v>0.884</v>
+      </c>
+      <c r="I67" s="4" t="n">
+        <v>0.885</v>
+      </c>
+      <c r="J67" s="4" t="n">
+        <v>0.886</v>
+      </c>
+      <c r="K67" s="4" t="n">
+        <v>0.887</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B68" s="3" t="n">
+        <v>0.8784</v>
+      </c>
+      <c r="C68" s="3" t="n">
+        <v>0.8794</v>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>0.8804</v>
+      </c>
+      <c r="E68" s="3" t="n">
+        <v>0.8813</v>
+      </c>
+      <c r="F68" s="3" t="n">
+        <v>0.8823</v>
+      </c>
+      <c r="G68" s="3" t="n">
+        <v>0.8833</v>
+      </c>
+      <c r="H68" s="3" t="n">
+        <v>0.8843</v>
+      </c>
+      <c r="I68" s="3" t="n">
+        <v>0.8853</v>
+      </c>
+      <c r="J68" s="3" t="n">
+        <v>0.8863</v>
+      </c>
+      <c r="K68" s="3" t="n">
+        <v>0.8873</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>33.5</v>
+      </c>
+      <c r="B69" s="4" t="n">
+        <v>0.8787</v>
+      </c>
+      <c r="C69" s="4" t="n">
+        <v>0.8797</v>
+      </c>
+      <c r="D69" s="4" t="n">
+        <v>0.8807</v>
+      </c>
+      <c r="E69" s="4" t="n">
+        <v>0.8817</v>
+      </c>
+      <c r="F69" s="4" t="n">
+        <v>0.8827</v>
+      </c>
+      <c r="G69" s="4" t="n">
+        <v>0.8837</v>
+      </c>
+      <c r="H69" s="4" t="n">
+        <v>0.8847</v>
+      </c>
+      <c r="I69" s="4" t="n">
+        <v>0.8857</v>
+      </c>
+      <c r="J69" s="4" t="n">
+        <v>0.8866000000000001</v>
+      </c>
+      <c r="K69" s="4" t="n">
+        <v>0.8875999999999999</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B70" s="3" t="n">
+        <v>0.879</v>
+      </c>
+      <c r="C70" s="3" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>0.881</v>
+      </c>
+      <c r="E70" s="3" t="n">
+        <v>0.882</v>
+      </c>
+      <c r="F70" s="3" t="n">
+        <v>0.883</v>
+      </c>
+      <c r="G70" s="3" t="n">
+        <v>0.884</v>
+      </c>
+      <c r="H70" s="3" t="n">
+        <v>0.885</v>
+      </c>
+      <c r="I70" s="3" t="n">
+        <v>0.886</v>
+      </c>
+      <c r="J70" s="3" t="n">
+        <v>0.887</v>
+      </c>
+      <c r="K70" s="3" t="n">
+        <v>0.888</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="B71" s="4" t="n">
+        <v>0.8793</v>
+      </c>
+      <c r="C71" s="4" t="n">
+        <v>0.8803</v>
+      </c>
+      <c r="D71" s="4" t="n">
+        <v>0.8813</v>
+      </c>
+      <c r="E71" s="4" t="n">
+        <v>0.8823</v>
+      </c>
+      <c r="F71" s="4" t="n">
+        <v>0.8833</v>
+      </c>
+      <c r="G71" s="4" t="n">
+        <v>0.8843</v>
+      </c>
+      <c r="H71" s="4" t="n">
+        <v>0.8853</v>
+      </c>
+      <c r="I71" s="4" t="n">
+        <v>0.8863</v>
+      </c>
+      <c r="J71" s="4" t="n">
+        <v>0.8873</v>
+      </c>
+      <c r="K71" s="4" t="n">
+        <v>0.8883</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B72" s="3" t="n">
+        <v>0.8796</v>
+      </c>
+      <c r="C72" s="3" t="n">
+        <v>0.8806</v>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>0.8816000000000001</v>
+      </c>
+      <c r="E72" s="3" t="n">
+        <v>0.8826000000000001</v>
+      </c>
+      <c r="F72" s="3" t="n">
+        <v>0.8836000000000001</v>
+      </c>
+      <c r="G72" s="3" t="n">
+        <v>0.8846000000000001</v>
+      </c>
+      <c r="H72" s="3" t="n">
+        <v>0.8856000000000001</v>
+      </c>
+      <c r="I72" s="3" t="n">
+        <v>0.8866000000000001</v>
+      </c>
+      <c r="J72" s="3" t="n">
+        <v>0.8875999999999999</v>
+      </c>
+      <c r="K72" s="3" t="n">
+        <v>0.8885999999999999</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>35.5</v>
+      </c>
+      <c r="B73" s="4" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="C73" s="4" t="n">
+        <v>0.881</v>
+      </c>
+      <c r="D73" s="4" t="n">
+        <v>0.8819</v>
+      </c>
+      <c r="E73" s="4" t="n">
+        <v>0.8829</v>
+      </c>
+      <c r="F73" s="4" t="n">
+        <v>0.8839</v>
+      </c>
+      <c r="G73" s="4" t="n">
+        <v>0.8849</v>
+      </c>
+      <c r="H73" s="4" t="n">
+        <v>0.8859</v>
+      </c>
+      <c r="I73" s="4" t="n">
+        <v>0.8869</v>
+      </c>
+      <c r="J73" s="4" t="n">
+        <v>0.8879</v>
+      </c>
+      <c r="K73" s="4" t="n">
+        <v>0.8889</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B74" s="3" t="n">
+        <v>0.8803</v>
+      </c>
+      <c r="C74" s="3" t="n">
+        <v>0.8813</v>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>0.8823</v>
+      </c>
+      <c r="E74" s="3" t="n">
+        <v>0.8833</v>
+      </c>
+      <c r="F74" s="3" t="n">
+        <v>0.8842</v>
+      </c>
+      <c r="G74" s="3" t="n">
+        <v>0.8852</v>
+      </c>
+      <c r="H74" s="3" t="n">
+        <v>0.8862</v>
+      </c>
+      <c r="I74" s="3" t="n">
+        <v>0.8872</v>
+      </c>
+      <c r="J74" s="3" t="n">
+        <v>0.8882</v>
+      </c>
+      <c r="K74" s="3" t="n">
+        <v>0.8892</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>36.5</v>
+      </c>
+      <c r="B75" s="4" t="n">
+        <v>0.8806</v>
+      </c>
+      <c r="C75" s="4" t="n">
+        <v>0.8816000000000001</v>
+      </c>
+      <c r="D75" s="4" t="n">
+        <v>0.8826000000000001</v>
+      </c>
+      <c r="E75" s="4" t="n">
+        <v>0.8836000000000001</v>
+      </c>
+      <c r="F75" s="4" t="n">
+        <v>0.8846000000000001</v>
+      </c>
+      <c r="G75" s="4" t="n">
+        <v>0.8856000000000001</v>
+      </c>
+      <c r="H75" s="4" t="n">
+        <v>0.8866000000000001</v>
+      </c>
+      <c r="I75" s="4" t="n">
+        <v>0.8875</v>
+      </c>
+      <c r="J75" s="4" t="n">
+        <v>0.8885</v>
+      </c>
+      <c r="K75" s="4" t="n">
+        <v>0.8895</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B76" s="3" t="n">
+        <v>0.8809</v>
+      </c>
+      <c r="C76" s="3" t="n">
+        <v>0.8819</v>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>0.8829</v>
+      </c>
+      <c r="E76" s="3" t="n">
+        <v>0.8839</v>
+      </c>
+      <c r="F76" s="3" t="n">
+        <v>0.8849</v>
+      </c>
+      <c r="G76" s="3" t="n">
+        <v>0.8859</v>
+      </c>
+      <c r="H76" s="3" t="n">
+        <v>0.8869</v>
+      </c>
+      <c r="I76" s="3" t="n">
+        <v>0.8879</v>
+      </c>
+      <c r="J76" s="3" t="n">
+        <v>0.8889</v>
+      </c>
+      <c r="K76" s="3" t="n">
+        <v>0.8899</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="B77" s="4" t="n">
+        <v>0.8812</v>
+      </c>
+      <c r="C77" s="4" t="n">
+        <v>0.8822</v>
+      </c>
+      <c r="D77" s="4" t="n">
+        <v>0.8832</v>
+      </c>
+      <c r="E77" s="4" t="n">
+        <v>0.8842</v>
+      </c>
+      <c r="F77" s="4" t="n">
+        <v>0.8852</v>
+      </c>
+      <c r="G77" s="4" t="n">
+        <v>0.8862</v>
+      </c>
+      <c r="H77" s="4" t="n">
+        <v>0.8872</v>
+      </c>
+      <c r="I77" s="4" t="n">
+        <v>0.8882</v>
+      </c>
+      <c r="J77" s="4" t="n">
+        <v>0.8892</v>
+      </c>
+      <c r="K77" s="4" t="n">
+        <v>0.8902</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="B78" s="3" t="n">
+        <v>0.8815</v>
+      </c>
+      <c r="C78" s="3" t="n">
+        <v>0.8825</v>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>0.8835</v>
+      </c>
+      <c r="E78" s="3" t="n">
+        <v>0.8845</v>
+      </c>
+      <c r="F78" s="3" t="n">
+        <v>0.8855</v>
+      </c>
+      <c r="G78" s="3" t="n">
+        <v>0.8865</v>
+      </c>
+      <c r="H78" s="3" t="n">
+        <v>0.8875</v>
+      </c>
+      <c r="I78" s="3" t="n">
+        <v>0.8885</v>
+      </c>
+      <c r="J78" s="3" t="n">
+        <v>0.8895</v>
+      </c>
+      <c r="K78" s="3" t="n">
+        <v>0.8905</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="B79" s="4" t="n">
+        <v>0.8819</v>
+      </c>
+      <c r="C79" s="4" t="n">
+        <v>0.8829</v>
+      </c>
+      <c r="D79" s="4" t="n">
+        <v>0.8838</v>
+      </c>
+      <c r="E79" s="4" t="n">
+        <v>0.8848</v>
+      </c>
+      <c r="F79" s="4" t="n">
+        <v>0.8858</v>
+      </c>
+      <c r="G79" s="4" t="n">
+        <v>0.8868</v>
+      </c>
+      <c r="H79" s="4" t="n">
+        <v>0.8878</v>
+      </c>
+      <c r="I79" s="4" t="n">
+        <v>0.8888</v>
+      </c>
+      <c r="J79" s="4" t="n">
+        <v>0.8898</v>
+      </c>
+      <c r="K79" s="4" t="n">
+        <v>0.8908</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B80" s="3" t="n">
+        <v>0.8822</v>
+      </c>
+      <c r="C80" s="3" t="n">
+        <v>0.8832</v>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>0.8842</v>
+      </c>
+      <c r="E80" s="3" t="n">
+        <v>0.8852</v>
+      </c>
+      <c r="F80" s="3" t="n">
+        <v>0.8862</v>
+      </c>
+      <c r="G80" s="3" t="n">
+        <v>0.8871</v>
+      </c>
+      <c r="H80" s="3" t="n">
+        <v>0.8881</v>
+      </c>
+      <c r="I80" s="3" t="n">
+        <v>0.8891</v>
+      </c>
+      <c r="J80" s="3" t="n">
+        <v>0.8901</v>
+      </c>
+      <c r="K80" s="3" t="n">
+        <v>0.8911</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>39.5</v>
+      </c>
+      <c r="B81" s="4" t="n">
+        <v>0.8825</v>
+      </c>
+      <c r="C81" s="4" t="n">
+        <v>0.8835</v>
+      </c>
+      <c r="D81" s="4" t="n">
+        <v>0.8845</v>
+      </c>
+      <c r="E81" s="4" t="n">
+        <v>0.8855</v>
+      </c>
+      <c r="F81" s="4" t="n">
+        <v>0.8865</v>
+      </c>
+      <c r="G81" s="4" t="n">
+        <v>0.8875</v>
+      </c>
+      <c r="H81" s="4" t="n">
+        <v>0.8885</v>
+      </c>
+      <c r="I81" s="4" t="n">
+        <v>0.8894</v>
+      </c>
+      <c r="J81" s="4" t="n">
+        <v>0.8904</v>
+      </c>
+      <c r="K81" s="4" t="n">
+        <v>0.8914</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="B82" s="3" t="n">
+        <v>0.8828</v>
+      </c>
+      <c r="C82" s="3" t="n">
+        <v>0.8838</v>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>0.8848</v>
+      </c>
+      <c r="E82" s="3" t="n">
+        <v>0.8858</v>
+      </c>
+      <c r="F82" s="3" t="n">
+        <v>0.8868</v>
+      </c>
+      <c r="G82" s="3" t="n">
+        <v>0.8878</v>
+      </c>
+      <c r="H82" s="3" t="n">
+        <v>0.8888</v>
+      </c>
+      <c r="I82" s="3" t="n">
+        <v>0.8898</v>
+      </c>
+      <c r="J82" s="3" t="n">
+        <v>0.8908</v>
+      </c>
+      <c r="K82" s="3" t="n">
+        <v>0.8917</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>40.5</v>
+      </c>
+      <c r="B83" s="4" t="n">
+        <v>0.8831</v>
+      </c>
+      <c r="C83" s="4" t="n">
+        <v>0.8841</v>
+      </c>
+      <c r="D83" s="4" t="n">
+        <v>0.8851</v>
+      </c>
+      <c r="E83" s="4" t="n">
+        <v>0.8861</v>
+      </c>
+      <c r="F83" s="4" t="n">
+        <v>0.8871</v>
+      </c>
+      <c r="G83" s="4" t="n">
+        <v>0.8881</v>
+      </c>
+      <c r="H83" s="4" t="n">
+        <v>0.8891</v>
+      </c>
+      <c r="I83" s="4" t="n">
+        <v>0.8901</v>
+      </c>
+      <c r="J83" s="4" t="n">
+        <v>0.8911</v>
+      </c>
+      <c r="K83" s="4" t="n">
+        <v>0.8921</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B84" s="3" t="n">
+        <v>0.8834</v>
+      </c>
+      <c r="C84" s="3" t="n">
+        <v>0.8844</v>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>0.8854</v>
+      </c>
+      <c r="E84" s="3" t="n">
+        <v>0.8864</v>
+      </c>
+      <c r="F84" s="3" t="n">
+        <v>0.8874</v>
+      </c>
+      <c r="G84" s="3" t="n">
+        <v>0.8884</v>
+      </c>
+      <c r="H84" s="3" t="n">
+        <v>0.8894</v>
+      </c>
+      <c r="I84" s="3" t="n">
+        <v>0.8904</v>
+      </c>
+      <c r="J84" s="3" t="n">
+        <v>0.8914</v>
+      </c>
+      <c r="K84" s="3" t="n">
+        <v>0.8924</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>41.5</v>
+      </c>
+      <c r="B85" s="4" t="n">
+        <v>0.8838</v>
+      </c>
+      <c r="C85" s="4" t="n">
+        <v>0.8848</v>
+      </c>
+      <c r="D85" s="4" t="n">
+        <v>0.8857</v>
+      </c>
+      <c r="E85" s="4" t="n">
+        <v>0.8867</v>
+      </c>
+      <c r="F85" s="4" t="n">
+        <v>0.8877</v>
+      </c>
+      <c r="G85" s="4" t="n">
+        <v>0.8887</v>
+      </c>
+      <c r="H85" s="4" t="n">
+        <v>0.8897</v>
+      </c>
+      <c r="I85" s="4" t="n">
+        <v>0.8907</v>
+      </c>
+      <c r="J85" s="4" t="n">
+        <v>0.8917</v>
+      </c>
+      <c r="K85" s="4" t="n">
+        <v>0.8927</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="B86" s="3" t="n">
+        <v>0.8841</v>
+      </c>
+      <c r="C86" s="3" t="n">
+        <v>0.8851</v>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>0.8861</v>
+      </c>
+      <c r="E86" s="3" t="n">
+        <v>0.8871</v>
+      </c>
+      <c r="F86" s="3" t="n">
+        <v>0.888</v>
+      </c>
+      <c r="G86" s="3" t="n">
+        <v>0.889</v>
+      </c>
+      <c r="H86" s="3" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="I86" s="3" t="n">
+        <v>0.891</v>
+      </c>
+      <c r="J86" s="3" t="n">
+        <v>0.892</v>
+      </c>
+      <c r="K86" s="3" t="n">
+        <v>0.893</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="B87" s="4" t="n">
+        <v>0.8844</v>
+      </c>
+      <c r="C87" s="4" t="n">
+        <v>0.8854</v>
+      </c>
+      <c r="D87" s="4" t="n">
+        <v>0.8864</v>
+      </c>
+      <c r="E87" s="4" t="n">
+        <v>0.8874</v>
+      </c>
+      <c r="F87" s="4" t="n">
+        <v>0.8884</v>
+      </c>
+      <c r="G87" s="4" t="n">
+        <v>0.8894</v>
+      </c>
+      <c r="H87" s="4" t="n">
+        <v>0.8903</v>
+      </c>
+      <c r="I87" s="4" t="n">
+        <v>0.8913</v>
+      </c>
+      <c r="J87" s="4" t="n">
+        <v>0.8923</v>
+      </c>
+      <c r="K87" s="4" t="n">
+        <v>0.8933</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="B88" s="3" t="n">
+        <v>0.8847</v>
+      </c>
+      <c r="C88" s="3" t="n">
+        <v>0.8857</v>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>0.8867</v>
+      </c>
+      <c r="E88" s="3" t="n">
+        <v>0.8877</v>
+      </c>
+      <c r="F88" s="3" t="n">
+        <v>0.8887</v>
+      </c>
+      <c r="G88" s="3" t="n">
+        <v>0.8897</v>
+      </c>
+      <c r="H88" s="3" t="n">
+        <v>0.8907</v>
+      </c>
+      <c r="I88" s="3" t="n">
+        <v>0.8915999999999999</v>
+      </c>
+      <c r="J88" s="3" t="n">
+        <v>0.8925999999999999</v>
+      </c>
+      <c r="K88" s="3" t="n">
+        <v>0.8935999999999999</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="B89" s="4" t="n">
+        <v>0.885</v>
+      </c>
+      <c r="C89" s="4" t="n">
+        <v>0.886</v>
+      </c>
+      <c r="D89" s="4" t="n">
+        <v>0.887</v>
+      </c>
+      <c r="E89" s="4" t="n">
+        <v>0.888</v>
+      </c>
+      <c r="F89" s="4" t="n">
+        <v>0.889</v>
+      </c>
+      <c r="G89" s="4" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="H89" s="4" t="n">
+        <v>0.891</v>
+      </c>
+      <c r="I89" s="4" t="n">
+        <v>0.892</v>
+      </c>
+      <c r="J89" s="4" t="n">
+        <v>0.893</v>
+      </c>
+      <c r="K89" s="4" t="n">
+        <v>0.8939</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="B90" s="3" t="n">
+        <v>0.8853</v>
+      </c>
+      <c r="C90" s="3" t="n">
+        <v>0.8863</v>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>0.8873</v>
+      </c>
+      <c r="E90" s="3" t="n">
+        <v>0.8883</v>
+      </c>
+      <c r="F90" s="3" t="n">
+        <v>0.8893</v>
+      </c>
+      <c r="G90" s="3" t="n">
+        <v>0.8903</v>
+      </c>
+      <c r="H90" s="3" t="n">
+        <v>0.8913</v>
+      </c>
+      <c r="I90" s="3" t="n">
+        <v>0.8923</v>
+      </c>
+      <c r="J90" s="3" t="n">
+        <v>0.8933</v>
+      </c>
+      <c r="K90" s="3" t="n">
+        <v>0.8943</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="B91" s="4" t="n">
+        <v>0.8857</v>
+      </c>
+      <c r="C91" s="4" t="n">
+        <v>0.8866000000000001</v>
+      </c>
+      <c r="D91" s="4" t="n">
+        <v>0.8875999999999999</v>
+      </c>
+      <c r="E91" s="4" t="n">
+        <v>0.8885999999999999</v>
+      </c>
+      <c r="F91" s="4" t="n">
+        <v>0.8895999999999999</v>
+      </c>
+      <c r="G91" s="4" t="n">
+        <v>0.8905999999999999</v>
+      </c>
+      <c r="H91" s="4" t="n">
+        <v>0.8915999999999999</v>
+      </c>
+      <c r="I91" s="4" t="n">
+        <v>0.8925999999999999</v>
+      </c>
+      <c r="J91" s="4" t="n">
+        <v>0.8935999999999999</v>
+      </c>
+      <c r="K91" s="4" t="n">
+        <v>0.8946</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="B92" s="3" t="n">
+        <v>0.886</v>
+      </c>
+      <c r="C92" s="3" t="n">
+        <v>0.887</v>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>0.8879</v>
+      </c>
+      <c r="E92" s="3" t="n">
+        <v>0.8889</v>
+      </c>
+      <c r="F92" s="3" t="n">
+        <v>0.8899</v>
+      </c>
+      <c r="G92" s="3" t="n">
+        <v>0.8909</v>
+      </c>
+      <c r="H92" s="3" t="n">
+        <v>0.8919</v>
+      </c>
+      <c r="I92" s="3" t="n">
+        <v>0.8929</v>
+      </c>
+      <c r="J92" s="3" t="n">
+        <v>0.8939</v>
+      </c>
+      <c r="K92" s="3" t="n">
+        <v>0.8949</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="B93" s="4" t="n">
+        <v>0.8863</v>
+      </c>
+      <c r="C93" s="4" t="n">
+        <v>0.8873</v>
+      </c>
+      <c r="D93" s="4" t="n">
+        <v>0.8883</v>
+      </c>
+      <c r="E93" s="4" t="n">
+        <v>0.8893</v>
+      </c>
+      <c r="F93" s="4" t="n">
+        <v>0.8902</v>
+      </c>
+      <c r="G93" s="4" t="n">
+        <v>0.8912</v>
+      </c>
+      <c r="H93" s="4" t="n">
+        <v>0.8922</v>
+      </c>
+      <c r="I93" s="4" t="n">
+        <v>0.8932</v>
+      </c>
+      <c r="J93" s="4" t="n">
+        <v>0.8942</v>
+      </c>
+      <c r="K93" s="4" t="n">
+        <v>0.8952</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="B94" s="3" t="n">
+        <v>0.8866000000000001</v>
+      </c>
+      <c r="C94" s="3" t="n">
+        <v>0.8875999999999999</v>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>0.8885999999999999</v>
+      </c>
+      <c r="E94" s="3" t="n">
+        <v>0.8895999999999999</v>
+      </c>
+      <c r="F94" s="3" t="n">
+        <v>0.8905999999999999</v>
+      </c>
+      <c r="G94" s="3" t="n">
+        <v>0.8915</v>
+      </c>
+      <c r="H94" s="3" t="n">
+        <v>0.8925</v>
+      </c>
+      <c r="I94" s="3" t="n">
+        <v>0.8935</v>
+      </c>
+      <c r="J94" s="3" t="n">
+        <v>0.8945</v>
+      </c>
+      <c r="K94" s="3" t="n">
+        <v>0.8955</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="B95" s="4" t="n">
+        <v>0.8869</v>
+      </c>
+      <c r="C95" s="4" t="n">
+        <v>0.8879</v>
+      </c>
+      <c r="D95" s="4" t="n">
+        <v>0.8889</v>
+      </c>
+      <c r="E95" s="4" t="n">
+        <v>0.8899</v>
+      </c>
+      <c r="F95" s="4" t="n">
+        <v>0.8909</v>
+      </c>
+      <c r="G95" s="4" t="n">
+        <v>0.8919</v>
+      </c>
+      <c r="H95" s="4" t="n">
+        <v>0.8929</v>
+      </c>
+      <c r="I95" s="4" t="n">
+        <v>0.8938</v>
+      </c>
+      <c r="J95" s="4" t="n">
+        <v>0.8948</v>
+      </c>
+      <c r="K95" s="4" t="n">
+        <v>0.8958</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="B96" s="3" t="n">
+        <v>0.8872</v>
+      </c>
+      <c r="C96" s="3" t="n">
+        <v>0.8882</v>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>0.8892</v>
+      </c>
+      <c r="E96" s="3" t="n">
+        <v>0.8902</v>
+      </c>
+      <c r="F96" s="3" t="n">
+        <v>0.8912</v>
+      </c>
+      <c r="G96" s="3" t="n">
+        <v>0.8922</v>
+      </c>
+      <c r="H96" s="3" t="n">
+        <v>0.8932</v>
+      </c>
+      <c r="I96" s="3" t="n">
+        <v>0.8942</v>
+      </c>
+      <c r="J96" s="3" t="n">
+        <v>0.8951</v>
+      </c>
+      <c r="K96" s="3" t="n">
+        <v>0.8961</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="B97" s="4" t="n">
+        <v>0.8875</v>
+      </c>
+      <c r="C97" s="4" t="n">
+        <v>0.8885</v>
+      </c>
+      <c r="D97" s="4" t="n">
+        <v>0.8895</v>
+      </c>
+      <c r="E97" s="4" t="n">
+        <v>0.8905</v>
+      </c>
+      <c r="F97" s="4" t="n">
+        <v>0.8915</v>
+      </c>
+      <c r="G97" s="4" t="n">
+        <v>0.8925</v>
+      </c>
+      <c r="H97" s="4" t="n">
+        <v>0.8935</v>
+      </c>
+      <c r="I97" s="4" t="n">
+        <v>0.8945</v>
+      </c>
+      <c r="J97" s="4" t="n">
+        <v>0.8954</v>
+      </c>
+      <c r="K97" s="4" t="n">
+        <v>0.8964</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="B98" s="3" t="n">
+        <v>0.8879</v>
+      </c>
+      <c r="C98" s="3" t="n">
+        <v>0.8888</v>
+      </c>
+      <c r="D98" s="3" t="n">
+        <v>0.8898</v>
+      </c>
+      <c r="E98" s="3" t="n">
+        <v>0.8908</v>
+      </c>
+      <c r="F98" s="3" t="n">
+        <v>0.8918</v>
+      </c>
+      <c r="G98" s="3" t="n">
+        <v>0.8928</v>
+      </c>
+      <c r="H98" s="3" t="n">
+        <v>0.8938</v>
+      </c>
+      <c r="I98" s="3" t="n">
+        <v>0.8948</v>
+      </c>
+      <c r="J98" s="3" t="n">
+        <v>0.8958</v>
+      </c>
+      <c r="K98" s="3" t="n">
+        <v>0.8967000000000001</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="B99" s="4" t="n">
+        <v>0.8882</v>
+      </c>
+      <c r="C99" s="4" t="n">
+        <v>0.8892</v>
+      </c>
+      <c r="D99" s="4" t="n">
+        <v>0.8901</v>
+      </c>
+      <c r="E99" s="4" t="n">
+        <v>0.8911</v>
+      </c>
+      <c r="F99" s="4" t="n">
+        <v>0.8921</v>
+      </c>
+      <c r="G99" s="4" t="n">
+        <v>0.8931</v>
+      </c>
+      <c r="H99" s="4" t="n">
+        <v>0.8941</v>
+      </c>
+      <c r="I99" s="4" t="n">
+        <v>0.8951</v>
+      </c>
+      <c r="J99" s="4" t="n">
+        <v>0.8961</v>
+      </c>
+      <c r="K99" s="4" t="n">
+        <v>0.8971</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="B100" s="3" t="n">
+        <v>0.8885</v>
+      </c>
+      <c r="C100" s="3" t="n">
+        <v>0.8895</v>
+      </c>
+      <c r="D100" s="3" t="n">
+        <v>0.8905</v>
+      </c>
+      <c r="E100" s="3" t="n">
+        <v>0.8914</v>
+      </c>
+      <c r="F100" s="3" t="n">
+        <v>0.8924</v>
+      </c>
+      <c r="G100" s="3" t="n">
+        <v>0.8934</v>
+      </c>
+      <c r="H100" s="3" t="n">
+        <v>0.8944</v>
+      </c>
+      <c r="I100" s="3" t="n">
+        <v>0.8954</v>
+      </c>
+      <c r="J100" s="3" t="n">
+        <v>0.8964</v>
+      </c>
+      <c r="K100" s="3" t="n">
+        <v>0.8974</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="n">
+        <v>49.5</v>
+      </c>
+      <c r="B101" s="4" t="n">
+        <v>0.8888</v>
+      </c>
+      <c r="C101" s="4" t="n">
+        <v>0.8898</v>
+      </c>
+      <c r="D101" s="4" t="n">
+        <v>0.8908</v>
+      </c>
+      <c r="E101" s="4" t="n">
+        <v>0.8917</v>
+      </c>
+      <c r="F101" s="4" t="n">
+        <v>0.8927</v>
+      </c>
+      <c r="G101" s="4" t="n">
+        <v>0.8937</v>
+      </c>
+      <c r="H101" s="4" t="n">
+        <v>0.8947000000000001</v>
+      </c>
+      <c r="I101" s="4" t="n">
+        <v>0.8957000000000001</v>
+      </c>
+      <c r="J101" s="4" t="n">
+        <v>0.8967000000000001</v>
+      </c>
+      <c r="K101" s="4" t="n">
+        <v>0.8977000000000001</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="B102" s="3" t="n">
+        <v>0.8891</v>
+      </c>
+      <c r="C102" s="3" t="n">
+        <v>0.8901</v>
+      </c>
+      <c r="D102" s="3" t="n">
+        <v>0.8911</v>
+      </c>
+      <c r="E102" s="3" t="n">
+        <v>0.8921</v>
+      </c>
+      <c r="F102" s="3" t="n">
+        <v>0.8931</v>
+      </c>
+      <c r="G102" s="3" t="n">
+        <v>0.894</v>
+      </c>
+      <c r="H102" s="3" t="n">
+        <v>0.895</v>
+      </c>
+      <c r="I102" s="3" t="n">
+        <v>0.896</v>
+      </c>
+      <c r="J102" s="3" t="n">
+        <v>0.897</v>
+      </c>
+      <c r="K102" s="3" t="n">
+        <v>0.898</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>